<commit_message>
Preserve blank search policy cells in derived case workbooks
</commit_message>
<xml_diff>
--- a/cases/case_260915_ci_small/178A/config.xlsx
+++ b/cases/case_260915_ci_small/178A/config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R45e19ec59f7b4afe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R25b9808dcb154ae0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R7499641ae3db4731"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R5b640194525845b9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R01e128eb50b24bc4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R46243819ce66458f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="Rbcbaa53478684079"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R062edd6914d14758"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4966,10 +4966,7 @@
           <x:t xml:space="preserve">keep_top_n</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="21" t="b">
-        <x:f>TRUE()</x:f>
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="B9" s="21"/>
       <x:c r="C9" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -4990,14 +4987,8 @@
           <x:t xml:space="preserve">keep_all_rows</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="21" t="b">
-        <x:f>TRUE()</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C10" s="16" t="b">
-        <x:f>FALSE()</x:f>
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="B10" s="21"/>
+      <x:c r="C10" s="16"/>
       <x:c r="D10" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -5015,14 +5006,8 @@
           <x:t xml:space="preserve">continue_on_error</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="21" t="b">
-        <x:f>TRUE()</x:f>
-        <x:v>1</x:v>
-      </x:c>
-      <x:c r="C11" s="16" t="b">
-        <x:f>TRUE()</x:f>
-        <x:v>1</x:v>
-      </x:c>
+      <x:c r="B11" s="21"/>
+      <x:c r="C11" s="16"/>
       <x:c r="D11" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>

</xml_diff>

<commit_message>
Milestone: align 178A COM flow with SiCoPR reference
</commit_message>
<xml_diff>
--- a/cases/case_260915_ci_small/178A/config.xlsx
+++ b/cases/case_260915_ci_small/178A/config.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R01e128eb50b24bc4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R46243819ce66458f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="Rbcbaa53478684079"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R062edd6914d14758"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R8f2f85a171cc40e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R0335efe414334b1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R87f95a9484734de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="run_config" sheetId="4" r:id="R54e46831a0184872"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -170,7 +170,7 @@
     <x:xf/>
     <x:xf/>
   </x:cellStyleXfs>
-  <x:cellXfs count="22">
+  <x:cellXfs count="26">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <x:alignment horizontal="general" vertical="bottom"/>
     </x:xf>
@@ -234,6 +234,28 @@
     </x:xf>
     <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="33" applyAlignment="1">
       <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="33" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="164" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+      <x:extLst>
+        <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
+          <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
+        </x:ext>
+      </x:extLst>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="19">
@@ -318,6 +340,23 @@
     </x:indexedColors>
   </x:colors>
 </x:styleSheet>
+</file>
+
+<file path=xl/featurePropertyBag/featurePropertyBag.xml><?xml version="1.0" encoding="utf-8"?>
+<xfpb:FeaturePropertyBags xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag">
+  <xfpb:bag type="Checkbox"/>
+  <xfpb:bag type="XFControls">
+    <xfpb:bagId k="CellControl">0</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplement">
+    <xfpb:bagId k="XFControls">1</xfpb:bagId>
+  </xfpb:bag>
+  <xfpb:bag type="XFComplements" extRef="XFComplementsMapperExtRef">
+    <xfpb:a k="MappedFeaturePropertyBags">
+      <xfpb:bagId>2</xfpb:bagId>
+    </xfpb:a>
+  </xfpb:bag>
+</xfpb:FeaturePropertyBags>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1588,7 +1627,7 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D38" s="16"/>
+      <x:c r="D38" s="16" t="n"/>
       <x:c r="E38" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -2194,7 +2233,7 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D58" s="16"/>
+      <x:c r="D58" s="16" t="n"/>
       <x:c r="E58" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -2800,7 +2839,7 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D78" s="16"/>
+      <x:c r="D78" s="16" t="n"/>
       <x:c r="E78" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -3406,7 +3445,7 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D98" s="16"/>
+      <x:c r="D98" s="16" t="n"/>
       <x:c r="E98" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -4448,7 +4487,7 @@
       </x:c>
       <x:c r="B133" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dy_override</x:t>
+          <x:t xml:space="preserve">dy_rel_As</x:t>
         </x:is>
       </x:c>
       <x:c r="C133" s="20" t="inlineStr">
@@ -4456,15 +4495,17 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D133" s="16" t="n"/>
+      <x:c r="D133" s="16" t="n">
+        <x:v>0.001</x:v>
+      </x:c>
       <x:c r="E133" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">V</x:t>
+          <x:t xml:space="preserve">dimensionless</x:t>
         </x:is>
       </x:c>
       <x:c r="F133" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Blank means derive from A_s.</x:t>
+          <x:t xml:space="preserve">Project PMF numerical control.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4476,7 +4517,7 @@
       </x:c>
       <x:c r="B134" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dy_rel_As</x:t>
+          <x:t xml:space="preserve">dy_abs_max</x:t>
         </x:is>
       </x:c>
       <x:c r="C134" s="20" t="inlineStr">
@@ -4485,11 +4526,11 @@
         </x:is>
       </x:c>
       <x:c r="D134" s="16" t="n">
-        <x:v>0.001</x:v>
+        <x:v>1e-05</x:v>
       </x:c>
       <x:c r="E134" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dimensionless</x:t>
+          <x:t xml:space="preserve">V</x:t>
         </x:is>
       </x:c>
       <x:c r="F134" s="21" t="inlineStr">
@@ -4506,7 +4547,7 @@
       </x:c>
       <x:c r="B135" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dy_abs_max</x:t>
+          <x:t xml:space="preserve">tap_rel_As</x:t>
         </x:is>
       </x:c>
       <x:c r="C135" s="20" t="inlineStr">
@@ -4515,11 +4556,11 @@
         </x:is>
       </x:c>
       <x:c r="D135" s="16" t="n">
-        <x:v>1e-05</x:v>
+        <x:v>0.001</x:v>
       </x:c>
       <x:c r="E135" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">V</x:t>
+          <x:t xml:space="preserve">dimensionless</x:t>
         </x:is>
       </x:c>
       <x:c r="F135" s="21" t="inlineStr">
@@ -4536,7 +4577,7 @@
       </x:c>
       <x:c r="B136" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">tap_abs_th_override</x:t>
+          <x:t xml:space="preserve">keep_mass</x:t>
         </x:is>
       </x:c>
       <x:c r="C136" s="20" t="inlineStr">
@@ -4544,15 +4585,17 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D136" s="16" t="n"/>
+      <x:c r="D136" s="16" t="n">
+        <x:v>0.99999</x:v>
+      </x:c>
       <x:c r="E136" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">V</x:t>
+          <x:t xml:space="preserve">probability</x:t>
         </x:is>
       </x:c>
       <x:c r="F136" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Blank means derive from A_s.</x:t>
+          <x:t xml:space="preserve">Project PMF truncation control.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4564,7 +4607,7 @@
       </x:c>
       <x:c r="B137" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">tap_rel_As</x:t>
+          <x:t xml:space="preserve">gaussian_n_sigma</x:t>
         </x:is>
       </x:c>
       <x:c r="C137" s="20" t="inlineStr">
@@ -4573,28 +4616,28 @@
         </x:is>
       </x:c>
       <x:c r="D137" s="16" t="n">
-        <x:v>0.001</x:v>
+        <x:v>8</x:v>
       </x:c>
       <x:c r="E137" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dimensionless</x:t>
+          <x:t xml:space="preserve">sigma</x:t>
         </x:is>
       </x:c>
       <x:c r="F137" s="21" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Project PMF numerical control.</x:t>
+          <x:t xml:space="preserve">Project Gaussian PMF half span.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="138" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A138" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">pmf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B138" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">keep_mass</x:t>
+      <x:c r="A138" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mlsd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B138" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mlsd_enable</x:t>
         </x:is>
       </x:c>
       <x:c r="C138" s="20" t="inlineStr">
@@ -4602,29 +4645,29 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D138" s="16" t="n">
-        <x:v>0.99999</x:v>
-      </x:c>
-      <x:c r="E138" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">probability</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F138" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Project PMF truncation control.</x:t>
+      <x:c r="D138" s="20" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E138" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">boolean</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F138" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Enable the Annex 178A MLSD stage. Remains disabled until a spec-traceable MLSD profile is available.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="139" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A139" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">pmf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B139" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">gaussian_n_sigma</x:t>
+      <x:c r="A139" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mlsd</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="B139" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">mlsd_trunc_len</x:t>
         </x:is>
       </x:c>
       <x:c r="C139" s="20" t="inlineStr">
@@ -4632,17 +4675,15 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D139" s="16" t="n">
-        <x:v>8</x:v>
-      </x:c>
-      <x:c r="E139" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">sigma</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F139" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Project Gaussian PMF half span.</x:t>
+      <x:c r="D139" s="20" t="n"/>
+      <x:c r="E139" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">events</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="F139" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">Required positive truncation length when MLSD is enabled; leave blank while disabled.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4654,7 +4695,7 @@
       </x:c>
       <x:c r="B140" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mlsd_enable</x:t>
+          <x:t xml:space="preserve">delta_com_an</x:t>
         </x:is>
       </x:c>
       <x:c r="C140" s="20" t="inlineStr">
@@ -4662,17 +4703,15 @@
           <x:t xml:space="preserve">intrinsic</x:t>
         </x:is>
       </x:c>
-      <x:c r="D140" s="20" t="b">
-        <x:v>0</x:v>
-      </x:c>
+      <x:c r="D140" s="20" t="n"/>
       <x:c r="E140" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">boolean</x:t>
+          <x:t xml:space="preserve">dB</x:t>
         </x:is>
       </x:c>
       <x:c r="F140" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Enable the Annex 178A MLSD stage. Remains disabled until a spec-traceable MLSD profile is available.</x:t>
+          <x:t xml:space="preserve">Optional explicit Annex 178A added-noise target. Do not use an ad-hoc test value as a project setting.</x:t>
         </x:is>
       </x:c>
     </x:row>
@@ -4684,7 +4723,7 @@
       </x:c>
       <x:c r="B141" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mlsd_trunc_len</x:t>
+          <x:t xml:space="preserve">minimum_com_limit</x:t>
         </x:is>
       </x:c>
       <x:c r="C141" s="20" t="inlineStr">
@@ -4695,101 +4734,105 @@
       <x:c r="D141" s="20" t="n"/>
       <x:c r="E141" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">events</x:t>
+          <x:t xml:space="preserve">dB</x:t>
         </x:is>
       </x:c>
       <x:c r="F141" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Required positive truncation length when MLSD is enabled; leave blank while disabled.</x:t>
+          <x:t xml:space="preserve">Fallback minimum COM limit from the owning clause or annex when delta_com_an is not explicitly supplied.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="142">
       <x:c r="A142" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">mlsd</x:t>
+          <x:t xml:space="preserve">channel</x:t>
         </x:is>
       </x:c>
       <x:c r="B142" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">delta_com_an</x:t>
+          <x:t xml:space="preserve">missing_dc_policy</x:t>
         </x:is>
       </x:c>
       <x:c r="C142" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">intrinsic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D142" s="20" t="n"/>
+          <x:t xml:space="preserve">policy</x:t>
+        </x:is>
+      </x:c>
+      <x:c r="D142" s="20" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">skrf</x:t>
+        </x:is>
+      </x:c>
       <x:c r="E142" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">dB</x:t>
+          <x:t xml:space="preserve">enum</x:t>
         </x:is>
       </x:c>
       <x:c r="F142" s="20" t="inlineStr">
         <x:is>
-          <x:t xml:space="preserve">Optional explicit Annex 178A added-noise target. Do not use an ad-hoc test value as a project setting.</x:t>
+          <x:t xml:space="preserve">DC handling before channel-to-LinkSegment conversion.</x:t>
         </x:is>
       </x:c>
     </x:row>
     <x:row r="143">
-      <x:c r="A143" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">mlsd</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B143" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">minimum_com_limit</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C143" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">intrinsic</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D143" s="20" t="n"/>
-      <x:c r="E143" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">dB</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F143" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Fallback minimum COM limit from the owning clause or annex when delta_com_an is not explicitly supplied.</x:t>
-        </x:is>
+      <x:c r="A143" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+      <x:c r="B143" t="str">
+        <x:v>R_0</x:v>
+      </x:c>
+      <x:c r="C143" t="str">
+        <x:v>intrinsic</x:v>
+      </x:c>
+      <x:c r="D143" t="n">
+        <x:v>46.25</x:v>
+      </x:c>
+      <x:c r="E143" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="F143" t="str">
+        <x:v>Single-ended COM reference resistance used by channel and package models.</x:v>
       </x:c>
     </x:row>
     <x:row r="144">
-      <x:c r="A144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">channel</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">missing_dc_policy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">policy</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">skrf</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">enum</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F144" s="20" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">DC handling before channel-to-LinkSegment conversion.</x:t>
-        </x:is>
+      <x:c r="A144" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+      <x:c r="B144" t="str">
+        <x:v>R_d_tx</x:v>
+      </x:c>
+      <x:c r="C144" t="str">
+        <x:v>intrinsic</x:v>
+      </x:c>
+      <x:c r="D144" t="n">
+        <x:v>46.25</x:v>
+      </x:c>
+      <x:c r="E144" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="F144" t="str">
+        <x:v>TX die termination resistance from the selected TX package profile.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" t="str">
+        <x:v>channel</x:v>
+      </x:c>
+      <x:c r="B145" t="str">
+        <x:v>R_d_rx</x:v>
+      </x:c>
+      <x:c r="C145" t="str">
+        <x:v>intrinsic</x:v>
+      </x:c>
+      <x:c r="D145" t="n">
+        <x:v>46.25</x:v>
+      </x:c>
+      <x:c r="E145" t="str">
+        <x:v>ohm</x:v>
+      </x:c>
+      <x:c r="F145" t="str">
+        <x:v>RX die termination resistance from the selected RX package profile.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -4854,8 +4897,10 @@
       <x:c r="B4" s="21" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="str">
-        <x:v>0:0.02:0.02</x:v>
+      <x:c r="C4" s="16" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">0:0.02:0.02</x:t>
+        </x:is>
       </x:c>
       <x:c r="D4" s="21" t="inlineStr">
         <x:is>
@@ -4923,8 +4968,10 @@
       <x:c r="B7" s="21" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="16" t="str">
-        <x:v>-1:1:0</x:v>
+      <x:c r="C7" s="16" t="inlineStr">
+        <x:is>
+          <x:t xml:space="preserve">-1:1:0</x:t>
+        </x:is>
       </x:c>
       <x:c r="D7" s="21" t="inlineStr">
         <x:is>
@@ -4966,7 +5013,7 @@
           <x:t xml:space="preserve">keep_top_n</x:t>
         </x:is>
       </x:c>
-      <x:c r="B9" s="21"/>
+      <x:c r="B9" s="21" t="n"/>
       <x:c r="C9" s="16" t="n">
         <x:v>10</x:v>
       </x:c>
@@ -4987,8 +5034,8 @@
           <x:t xml:space="preserve">keep_all_rows</x:t>
         </x:is>
       </x:c>
-      <x:c r="B10" s="21"/>
-      <x:c r="C10" s="16"/>
+      <x:c r="B10" s="21" t="n"/>
+      <x:c r="C10" s="16" t="n"/>
       <x:c r="D10" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -5006,8 +5053,8 @@
           <x:t xml:space="preserve">continue_on_error</x:t>
         </x:is>
       </x:c>
-      <x:c r="B11" s="21"/>
-      <x:c r="C11" s="16"/>
+      <x:c r="B11" s="21" t="n"/>
+      <x:c r="C11" s="16" t="n"/>
       <x:c r="D11" s="21" t="inlineStr">
         <x:is>
           <x:t xml:space="preserve">boolean</x:t>
@@ -5039,6 +5086,7 @@
     <x:col min="6" max="7" width="18" style="11" customWidth="1"/>
     <x:col min="8" max="8" width="10" style="11" customWidth="1"/>
     <x:col min="9" max="9" width="34" style="11" customWidth="1"/>
+    <x:col min="6" max="6" width="42" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" s="12" customFormat="1" ht="17.350000381469727" customHeight="1">
@@ -5049,261 +5097,195 @@
       </x:c>
     </x:row>
     <x:row r="3" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Kind</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Index</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="C3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">S4P Path</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Port Order</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">R0 Ohm</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="F3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gamma Source</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="G3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Gamma Load</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="H3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Use</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="I3" s="14" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Description</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="4" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A4" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">victim</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B4" s="21" t="n">
+      <x:c r="A3" s="14" t="str">
+        <x:v>Kind</x:v>
+      </x:c>
+      <x:c r="B3" s="14" t="str">
+        <x:v>Index</x:v>
+      </x:c>
+      <x:c r="C3" s="14" t="str">
+        <x:v>S4P Path</x:v>
+      </x:c>
+      <x:c r="D3" s="14" t="str">
+        <x:v>Port Order</x:v>
+      </x:c>
+      <x:c r="E3" s="14" t="str">
+        <x:v>Use</x:v>
+      </x:c>
+      <x:c r="F3" s="14" t="str">
+        <x:v>Description</x:v>
+      </x:c>
+      <x:c r="G3" s="14"/>
+      <x:c r="H3" s="14"/>
+      <x:c r="I3" s="14"/>
+    </x:row>
+    <x:row r="4" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A4" s="23" t="str">
+        <x:v>victim</x:v>
+      </x:c>
+      <x:c r="B4" s="23" t="n">
         <x:v>0</x:v>
       </x:c>
-      <x:c r="C4" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_t.s4p</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D4" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0,2,1,3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E4" s="21" t="n">
-        <x:v>46.25</x:v>
-      </x:c>
-      <x:c r="F4" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G4" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H4" s="21" t="b">
+      <x:c r="C4" s="24" t="str">
+        <x:v>../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_t.s4p</x:v>
+      </x:c>
+      <x:c r="D4" s="23" t="str">
+        <x:v>0,2,1,3</x:v>
+      </x:c>
+      <x:c r="E4" s="25" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I4" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">PCB host NoSkew Ml36_20 THRU</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="5" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A5" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">next</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B5" s="21" t="n">
+      <x:c r="F4" s="23" t="str">
+        <x:v>PCB host NoSkew Ml36_20 THRU</x:v>
+      </x:c>
+      <x:c r="G4" s="21"/>
+      <x:c r="H4" s="21"/>
+      <x:c r="I4" s="21"/>
+    </x:row>
+    <x:row r="5" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A5" s="23" t="str">
+        <x:v>next</x:v>
+      </x:c>
+      <x:c r="B5" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C5" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_n1.s4p</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D5" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0,2,1,3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E5" s="21" t="n">
-        <x:v>46.25</x:v>
-      </x:c>
-      <x:c r="F5" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G5" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H5" s="21" t="b">
+      <x:c r="C5" s="24" t="str">
+        <x:v>../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_n1.s4p</x:v>
+      </x:c>
+      <x:c r="D5" s="23" t="str">
+        <x:v>0,2,1,3</x:v>
+      </x:c>
+      <x:c r="E5" s="25" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I5" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Power-sum NEXT; include once</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="6" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A6" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">fext</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="B6" s="21" t="n">
+      <x:c r="F5" s="23" t="str">
+        <x:v>Power-sum NEXT; include once</x:v>
+      </x:c>
+      <x:c r="G5" s="21"/>
+      <x:c r="H5" s="21"/>
+      <x:c r="I5" s="21"/>
+    </x:row>
+    <x:row r="6" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A6" s="23" t="str">
+        <x:v>fext</x:v>
+      </x:c>
+      <x:c r="B6" s="23" t="n">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="16" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_f1.s4p</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="D6" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0,2,1,3</x:t>
-        </x:is>
-      </x:c>
-      <x:c r="E6" s="21" t="n">
-        <x:v>46.25</x:v>
-      </x:c>
-      <x:c r="F6" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="G6" s="21" t="n">
-        <x:v>0</x:v>
-      </x:c>
-      <x:c r="H6" s="21" t="b">
+      <x:c r="C6" s="24" t="str">
+        <x:v>../../../reference_data/COM_channel_data/C2M/kareti_3dj_elec_02_240111/PCB_host/NoSkew/pcb_hst_S4_B2B_s0nl0_Ml36_20_f1.s4p</x:v>
+      </x:c>
+      <x:c r="D6" s="23" t="str">
+        <x:v>0,2,1,3</x:v>
+      </x:c>
+      <x:c r="E6" s="25" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="I6" s="21" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Power-sum FEXT; include once</x:t>
-        </x:is>
-      </x:c>
-    </x:row>
-    <x:row r="7" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A7" s="21" t="n"/>
-      <x:c r="B7" s="21" t="n"/>
-      <x:c r="C7" s="16" t="n"/>
-      <x:c r="D7" s="21" t="n"/>
-      <x:c r="E7" s="21" t="n"/>
-      <x:c r="F7" s="21" t="n"/>
-      <x:c r="G7" s="21" t="n"/>
-      <x:c r="H7" s="21" t="n"/>
-      <x:c r="I7" s="21" t="n"/>
-    </x:row>
-    <x:row r="8" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A8" s="21" t="n"/>
-      <x:c r="B8" s="21" t="n"/>
-      <x:c r="C8" s="16" t="n"/>
-      <x:c r="D8" s="21" t="n"/>
-      <x:c r="E8" s="21" t="n"/>
-      <x:c r="F8" s="21" t="n"/>
-      <x:c r="G8" s="21" t="n"/>
-      <x:c r="H8" s="21" t="n"/>
-      <x:c r="I8" s="21" t="n"/>
-    </x:row>
-    <x:row r="9" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A9" s="21" t="n"/>
-      <x:c r="B9" s="21" t="n"/>
-      <x:c r="C9" s="16" t="n"/>
-      <x:c r="D9" s="21" t="n"/>
-      <x:c r="E9" s="21" t="n"/>
-      <x:c r="F9" s="21" t="n"/>
-      <x:c r="G9" s="21" t="n"/>
-      <x:c r="H9" s="21" t="n"/>
-      <x:c r="I9" s="21" t="n"/>
-    </x:row>
-    <x:row r="10" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A10" s="21" t="n"/>
-      <x:c r="B10" s="21" t="n"/>
-      <x:c r="C10" s="16" t="n"/>
-      <x:c r="D10" s="21" t="n"/>
-      <x:c r="E10" s="21" t="n"/>
-      <x:c r="F10" s="21" t="n"/>
-      <x:c r="G10" s="21" t="n"/>
-      <x:c r="H10" s="21" t="n"/>
-      <x:c r="I10" s="21" t="n"/>
-    </x:row>
-    <x:row r="11" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A11" s="21" t="n"/>
-      <x:c r="B11" s="21" t="n"/>
-      <x:c r="C11" s="16" t="n"/>
-      <x:c r="D11" s="21" t="n"/>
-      <x:c r="E11" s="21" t="n"/>
-      <x:c r="F11" s="21" t="n"/>
-      <x:c r="G11" s="21" t="n"/>
-      <x:c r="H11" s="21" t="n"/>
-      <x:c r="I11" s="21" t="n"/>
-    </x:row>
-    <x:row r="12" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A12" s="21" t="n"/>
-      <x:c r="B12" s="21" t="n"/>
-      <x:c r="C12" s="16" t="n"/>
-      <x:c r="D12" s="21" t="n"/>
-      <x:c r="E12" s="21" t="n"/>
-      <x:c r="F12" s="21" t="n"/>
-      <x:c r="G12" s="21" t="n"/>
-      <x:c r="H12" s="21" t="n"/>
-      <x:c r="I12" s="21" t="n"/>
-    </x:row>
-    <x:row r="13" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A13" s="21" t="n"/>
-      <x:c r="B13" s="21" t="n"/>
-      <x:c r="C13" s="16" t="n"/>
-      <x:c r="D13" s="21" t="n"/>
-      <x:c r="E13" s="21" t="n"/>
-      <x:c r="F13" s="21" t="n"/>
-      <x:c r="G13" s="21" t="n"/>
-      <x:c r="H13" s="21" t="n"/>
-      <x:c r="I13" s="21" t="n"/>
-    </x:row>
-    <x:row r="14" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A14" s="21" t="n"/>
-      <x:c r="B14" s="21" t="n"/>
-      <x:c r="C14" s="16" t="n"/>
-      <x:c r="D14" s="21" t="n"/>
-      <x:c r="E14" s="21" t="n"/>
-      <x:c r="F14" s="21" t="n"/>
-      <x:c r="G14" s="21" t="n"/>
-      <x:c r="H14" s="21" t="n"/>
-      <x:c r="I14" s="21" t="n"/>
-    </x:row>
-    <x:row r="15" s="12" customFormat="1" ht="15" customHeight="1">
-      <x:c r="A15" s="21" t="n"/>
-      <x:c r="B15" s="21" t="n"/>
-      <x:c r="C15" s="16" t="n"/>
-      <x:c r="D15" s="21" t="n"/>
-      <x:c r="E15" s="21" t="n"/>
-      <x:c r="F15" s="21" t="n"/>
-      <x:c r="G15" s="21" t="n"/>
-      <x:c r="H15" s="21" t="n"/>
-      <x:c r="I15" s="21" t="n"/>
+      <x:c r="F6" s="23" t="str">
+        <x:v>Power-sum FEXT; include once</x:v>
+      </x:c>
+      <x:c r="G6" s="21"/>
+      <x:c r="H6" s="21"/>
+      <x:c r="I6" s="21"/>
+    </x:row>
+    <x:row r="7" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A7" s="23"/>
+      <x:c r="B7" s="23"/>
+      <x:c r="C7" s="24"/>
+      <x:c r="D7" s="23"/>
+      <x:c r="E7" s="23"/>
+      <x:c r="F7" s="23"/>
+      <x:c r="G7" s="21"/>
+      <x:c r="H7" s="21"/>
+      <x:c r="I7" s="21"/>
+    </x:row>
+    <x:row r="8" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A8" s="23"/>
+      <x:c r="B8" s="23"/>
+      <x:c r="C8" s="24"/>
+      <x:c r="D8" s="23"/>
+      <x:c r="E8" s="23"/>
+      <x:c r="F8" s="23"/>
+      <x:c r="G8" s="21"/>
+      <x:c r="H8" s="21"/>
+      <x:c r="I8" s="21"/>
+    </x:row>
+    <x:row r="9" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A9" s="23"/>
+      <x:c r="B9" s="23"/>
+      <x:c r="C9" s="24"/>
+      <x:c r="D9" s="23"/>
+      <x:c r="E9" s="23"/>
+      <x:c r="F9" s="23"/>
+      <x:c r="G9" s="21"/>
+      <x:c r="H9" s="21"/>
+      <x:c r="I9" s="21"/>
+    </x:row>
+    <x:row r="10" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A10" s="23"/>
+      <x:c r="B10" s="23"/>
+      <x:c r="C10" s="24"/>
+      <x:c r="D10" s="23"/>
+      <x:c r="E10" s="23"/>
+      <x:c r="F10" s="23"/>
+      <x:c r="G10" s="21"/>
+      <x:c r="H10" s="21"/>
+      <x:c r="I10" s="21"/>
+    </x:row>
+    <x:row r="11" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A11" s="23"/>
+      <x:c r="B11" s="23"/>
+      <x:c r="C11" s="24"/>
+      <x:c r="D11" s="23"/>
+      <x:c r="E11" s="23"/>
+      <x:c r="F11" s="23"/>
+      <x:c r="G11" s="21"/>
+      <x:c r="H11" s="21"/>
+      <x:c r="I11" s="21"/>
+    </x:row>
+    <x:row r="12" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A12" s="23"/>
+      <x:c r="B12" s="23"/>
+      <x:c r="C12" s="24"/>
+      <x:c r="D12" s="23"/>
+      <x:c r="E12" s="23"/>
+      <x:c r="F12" s="23"/>
+      <x:c r="G12" s="21"/>
+      <x:c r="H12" s="21"/>
+      <x:c r="I12" s="21"/>
+    </x:row>
+    <x:row r="13" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A13" s="23"/>
+      <x:c r="B13" s="23"/>
+      <x:c r="C13" s="24"/>
+      <x:c r="D13" s="23"/>
+      <x:c r="E13" s="23"/>
+      <x:c r="F13" s="23"/>
+      <x:c r="G13" s="21"/>
+      <x:c r="H13" s="21"/>
+      <x:c r="I13" s="21"/>
+    </x:row>
+    <x:row r="14" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A14" s="23"/>
+      <x:c r="B14" s="23"/>
+      <x:c r="C14" s="24"/>
+      <x:c r="D14" s="23"/>
+      <x:c r="E14" s="23"/>
+      <x:c r="F14" s="23"/>
+      <x:c r="G14" s="21"/>
+      <x:c r="H14" s="21"/>
+      <x:c r="I14" s="21"/>
+    </x:row>
+    <x:row r="15" s="12" customFormat="1" ht="30" customHeight="1">
+      <x:c r="A15" s="23"/>
+      <x:c r="B15" s="23"/>
+      <x:c r="C15" s="24"/>
+      <x:c r="D15" s="23"/>
+      <x:c r="E15" s="23"/>
+      <x:c r="F15" s="23"/>
+      <x:c r="G15" s="21"/>
+      <x:c r="H15" s="21"/>
+      <x:c r="I15" s="21"/>
     </x:row>
   </x:sheetData>
   <x:mergeCells>

</xml_diff>